<commit_message>
correções na planilha de indicadores
</commit_message>
<xml_diff>
--- a/data-raw/data_pfgp/plataforma_pfgp_indicadores 2.xlsx
+++ b/data-raw/data_pfgp/plataforma_pfgp_indicadores 2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wesley.jesus\Documents\PainelMonitoramento\data-raw\data_pfgp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E105638-DEBE-4819-9377-EA7A427859BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A92C01D-1C92-4AC5-9E4A-17D7A4D897E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{E40FA4F7-9C2D-425A-B6CE-BAADE3E52F77}"/>
   </bookViews>
@@ -20,6 +20,7 @@
     <sheet name="Planilha1" sheetId="5" r:id="rId5"/>
   </sheets>
   <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Indicadores PFGP'!$A$1:$AE$82</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Mapeamento informações'!$A$1:$I$106</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
@@ -46,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1904" uniqueCount="508">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1903" uniqueCount="508">
   <si>
     <t>id_indicador</t>
   </si>
@@ -7980,12 +7981,8 @@
         <v>1</v>
       </c>
       <c r="T39" s="19"/>
-      <c r="U39" s="31" t="s">
-        <v>17</v>
-      </c>
-      <c r="V39" s="19">
-        <v>1</v>
-      </c>
+      <c r="U39" s="31"/>
+      <c r="V39" s="19"/>
       <c r="W39" s="19"/>
       <c r="Z39" s="19"/>
       <c r="AA39" s="19"/>
@@ -12329,6 +12326,7 @@
       <c r="AE153" s="15"/>
     </row>
   </sheetData>
+  <autoFilter ref="A1:AE82" xr:uid="{120D1273-48A9-4A2C-B8BC-89F8F1D1C460}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:AE74">
     <sortCondition ref="A2:A74"/>
   </sortState>

</xml_diff>